<commit_message>
Fixed 08 - March 2026 close + Q1 Roll-Up
</commit_message>
<xml_diff>
--- a/submissions/excel/excel_08_march_close_q1.xlsx
+++ b/submissions/excel/excel_08_march_close_q1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venti\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7EC9421-85AF-4CA7-9B49-82B378415AE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4A4E1EB-A51D-44C1-ABB0-37EFA8A98DAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3540,7 +3540,7 @@
     <numFmt numFmtId="177" formatCode="mmm_yyyyy"/>
     <numFmt numFmtId="178" formatCode="&quot;$&quot;#,##0.00;\(&quot;$&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="179" formatCode="0.0%;\(0.0%\);\-"/>
-    <numFmt numFmtId="186" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="180" formatCode="0.00&quot;x&quot;"/>
   </numFmts>
   <fonts count="49" x14ac:knownFonts="1">
     <font>
@@ -4128,7 +4128,7 @@
     <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="219">
+  <cellXfs count="218">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4402,6 +4402,38 @@
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="48" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="178" fontId="39" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="178" fontId="40" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="179" fontId="39" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="170" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="170" fontId="36" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="36" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="36" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="36" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="29" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="36" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -4411,39 +4443,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="48" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="178" fontId="39" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="178" fontId="40" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="179" fontId="39" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="175" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="170" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="170" fontId="36" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="36" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="186" fontId="36" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="36" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -5223,7 +5222,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="1" width="525" row="7">
+  <wetp:taskpane dockstate="right" visibility="1" width="525" row="6">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -6478,30 +6477,30 @@
       <c r="A47" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B47" s="193" t="s">
+      <c r="B47" s="213" t="s">
         <v>311</v>
       </c>
-      <c r="C47" s="193"/>
-      <c r="D47" s="193"/>
-      <c r="E47" s="193"/>
-      <c r="F47" s="193"/>
-      <c r="G47" s="193"/>
-      <c r="H47" s="193"/>
-      <c r="I47" s="193"/>
+      <c r="C47" s="213"/>
+      <c r="D47" s="213"/>
+      <c r="E47" s="213"/>
+      <c r="F47" s="213"/>
+      <c r="G47" s="213"/>
+      <c r="H47" s="213"/>
+      <c r="I47" s="213"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B49" s="193" t="s">
+      <c r="B49" s="213" t="s">
         <v>312</v>
       </c>
-      <c r="C49" s="193"/>
-      <c r="D49" s="193"/>
-      <c r="E49" s="193"/>
-      <c r="F49" s="193"/>
-      <c r="G49" s="193"/>
-      <c r="H49" s="193"/>
+      <c r="C49" s="213"/>
+      <c r="D49" s="213"/>
+      <c r="E49" s="213"/>
+      <c r="F49" s="213"/>
+      <c r="G49" s="213"/>
+      <c r="H49" s="213"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -9924,35 +9923,35 @@
       </c>
     </row>
     <row r="34" spans="1:27" ht="80" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="195" t="s">
+      <c r="A34" s="215" t="s">
         <v>188</v>
       </c>
-      <c r="B34" s="196"/>
-      <c r="C34" s="196"/>
-      <c r="D34" s="196"/>
-      <c r="E34" s="196"/>
-      <c r="F34" s="196"/>
-      <c r="G34" s="196"/>
-      <c r="H34" s="196"/>
-      <c r="I34" s="196"/>
-      <c r="J34" s="196"/>
-      <c r="K34" s="196"/>
-      <c r="L34" s="196"/>
-      <c r="M34" s="196"/>
-      <c r="N34" s="196"/>
-      <c r="O34" s="196"/>
-      <c r="P34" s="196"/>
-      <c r="Q34" s="196"/>
-      <c r="R34" s="196"/>
-      <c r="S34" s="196"/>
-      <c r="T34" s="196"/>
-      <c r="U34" s="196"/>
-      <c r="V34" s="196"/>
-      <c r="W34" s="196"/>
-      <c r="X34" s="196"/>
-      <c r="Y34" s="196"/>
-      <c r="Z34" s="196"/>
-      <c r="AA34" s="196"/>
+      <c r="B34" s="216"/>
+      <c r="C34" s="216"/>
+      <c r="D34" s="216"/>
+      <c r="E34" s="216"/>
+      <c r="F34" s="216"/>
+      <c r="G34" s="216"/>
+      <c r="H34" s="216"/>
+      <c r="I34" s="216"/>
+      <c r="J34" s="216"/>
+      <c r="K34" s="216"/>
+      <c r="L34" s="216"/>
+      <c r="M34" s="216"/>
+      <c r="N34" s="216"/>
+      <c r="O34" s="216"/>
+      <c r="P34" s="216"/>
+      <c r="Q34" s="216"/>
+      <c r="R34" s="216"/>
+      <c r="S34" s="216"/>
+      <c r="T34" s="216"/>
+      <c r="U34" s="216"/>
+      <c r="V34" s="216"/>
+      <c r="W34" s="216"/>
+      <c r="X34" s="216"/>
+      <c r="Y34" s="216"/>
+      <c r="Z34" s="216"/>
+      <c r="AA34" s="216"/>
     </row>
     <row r="35" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="36" spans="1:27" x14ac:dyDescent="0.35">
@@ -9961,35 +9960,35 @@
       </c>
     </row>
     <row r="37" spans="1:27" ht="95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="195" t="s">
+      <c r="A37" s="215" t="s">
         <v>190</v>
       </c>
-      <c r="B37" s="196"/>
-      <c r="C37" s="196"/>
-      <c r="D37" s="196"/>
-      <c r="E37" s="196"/>
-      <c r="F37" s="196"/>
-      <c r="G37" s="196"/>
-      <c r="H37" s="196"/>
-      <c r="I37" s="196"/>
-      <c r="J37" s="196"/>
-      <c r="K37" s="196"/>
-      <c r="L37" s="196"/>
-      <c r="M37" s="196"/>
-      <c r="N37" s="196"/>
-      <c r="O37" s="196"/>
-      <c r="P37" s="196"/>
-      <c r="Q37" s="196"/>
-      <c r="R37" s="196"/>
-      <c r="S37" s="196"/>
-      <c r="T37" s="196"/>
-      <c r="U37" s="196"/>
-      <c r="V37" s="196"/>
-      <c r="W37" s="196"/>
-      <c r="X37" s="196"/>
-      <c r="Y37" s="196"/>
-      <c r="Z37" s="196"/>
-      <c r="AA37" s="196"/>
+      <c r="B37" s="216"/>
+      <c r="C37" s="216"/>
+      <c r="D37" s="216"/>
+      <c r="E37" s="216"/>
+      <c r="F37" s="216"/>
+      <c r="G37" s="216"/>
+      <c r="H37" s="216"/>
+      <c r="I37" s="216"/>
+      <c r="J37" s="216"/>
+      <c r="K37" s="216"/>
+      <c r="L37" s="216"/>
+      <c r="M37" s="216"/>
+      <c r="N37" s="216"/>
+      <c r="O37" s="216"/>
+      <c r="P37" s="216"/>
+      <c r="Q37" s="216"/>
+      <c r="R37" s="216"/>
+      <c r="S37" s="216"/>
+      <c r="T37" s="216"/>
+      <c r="U37" s="216"/>
+      <c r="V37" s="216"/>
+      <c r="W37" s="216"/>
+      <c r="X37" s="216"/>
+      <c r="Y37" s="216"/>
+      <c r="Z37" s="216"/>
+      <c r="AA37" s="216"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -10713,18 +10712,18 @@
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A64" s="197" t="s">
+      <c r="A64" s="217" t="s">
         <v>256</v>
       </c>
-      <c r="B64" s="197"/>
-      <c r="C64" s="197"/>
-      <c r="D64" s="197"/>
-      <c r="E64" s="197"/>
-      <c r="F64" s="197"/>
-      <c r="G64" s="197"/>
-      <c r="H64" s="197"/>
-      <c r="I64" s="197"/>
-      <c r="J64" s="197"/>
+      <c r="B64" s="217"/>
+      <c r="C64" s="217"/>
+      <c r="D64" s="217"/>
+      <c r="E64" s="217"/>
+      <c r="F64" s="217"/>
+      <c r="G64" s="217"/>
+      <c r="H64" s="217"/>
+      <c r="I64" s="217"/>
+      <c r="J64" s="217"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="62" t="s">
@@ -13701,7 +13700,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="128">
-        <v>180</v>
+        <v>380</v>
       </c>
       <c r="C5" s="128">
         <f>'2026 Forecast'!B9/3</f>
@@ -13709,11 +13708,11 @@
       </c>
       <c r="D5" s="128">
         <f t="shared" si="0"/>
-        <v>-535.34749999999997</v>
+        <v>-335.34749999999997</v>
       </c>
       <c r="E5" s="129">
         <f>IFERROR(B5/C5-1, 0)</f>
-        <v>-0.74837404198658697</v>
+        <v>-0.46878964419390579</v>
       </c>
       <c r="F5" s="130" t="str" cm="1">
         <f t="array" ref="F5">_xlfn.IFS(D5&lt;0, "U", D5&gt;0, "F", D5=0, "-")</f>
@@ -13773,7 +13772,7 @@
       </c>
       <c r="B8" s="135">
         <f>B4+B5-B7</f>
-        <v>3180</v>
+        <v>3380</v>
       </c>
       <c r="C8" s="135">
         <f>C4+C5-C7</f>
@@ -13781,11 +13780,11 @@
       </c>
       <c r="D8" s="135">
         <f t="shared" si="0"/>
-        <v>-581.55083333333323</v>
+        <v>-381.55083333333323</v>
       </c>
       <c r="E8" s="136">
         <f>B8/C8-1</f>
-        <v>-0.1546040075226065</v>
+        <v>-0.10143444824729864</v>
       </c>
       <c r="F8" s="137" t="str" cm="1">
         <f t="array" ref="F8">_xlfn.IFS(D8&lt;0, "U", D8&gt;0, "F", D8=0, "-")</f>
@@ -13798,7 +13797,7 @@
       </c>
       <c r="B9" s="139">
         <f>B3+B4+B5-B7</f>
-        <v>153485.5</v>
+        <v>153685.5</v>
       </c>
       <c r="C9" s="139">
         <f>C3+C8</f>
@@ -13806,11 +13805,11 @@
       </c>
       <c r="D9" s="139">
         <f t="shared" si="0"/>
-        <v>-868.65083333334769</v>
+        <v>-668.65083333334769</v>
       </c>
       <c r="E9" s="140">
         <f>B9/C9-1</f>
-        <v>-5.6276480330696987E-3</v>
+        <v>-4.3319264802624824E-3</v>
       </c>
       <c r="F9" s="141" t="str" cm="1">
         <f t="array" ref="F9">_xlfn.IFS(D9&lt;0, "U", D9&gt;0, "F", D9=0, "-")</f>
@@ -13823,7 +13822,7 @@
       </c>
       <c r="B10" s="142">
         <f>B9*12</f>
-        <v>1841826</v>
+        <v>1844226</v>
       </c>
       <c r="C10" s="142">
         <f>C9*12</f>
@@ -13831,11 +13830,11 @@
       </c>
       <c r="D10" s="142">
         <f t="shared" si="0"/>
-        <v>-10423.810000000056</v>
+        <v>-8023.8100000000559</v>
       </c>
       <c r="E10" s="143">
         <f>B10/C10-1</f>
-        <v>-5.6276480330695877E-3</v>
+        <v>-4.3319264802624824E-3</v>
       </c>
       <c r="F10" s="144" t="str" cm="1">
         <f t="array" ref="F10">_xlfn.IFS(D10&lt;0, "U", D10&gt;0, "F", D10=0, "-")</f>
@@ -13881,7 +13880,7 @@
       </c>
       <c r="B14" s="131">
         <f>B9</f>
-        <v>153485.5</v>
+        <v>153685.5</v>
       </c>
       <c r="C14" s="131">
         <f>C9</f>
@@ -13889,11 +13888,11 @@
       </c>
       <c r="D14" s="131">
         <f t="shared" ref="D14:D23" si="1">B14-C14</f>
-        <v>-868.65083333334769</v>
+        <v>-668.65083333334769</v>
       </c>
       <c r="E14" s="132">
         <f t="shared" ref="E14:E23" si="2">B14/C14-1</f>
-        <v>-5.6276480330696987E-3</v>
+        <v>-4.3319264802624824E-3</v>
       </c>
       <c r="F14" s="130" t="str" cm="1">
         <f t="array" ref="F14">_xlfn.IFS(D14&lt;0, "U", D14&gt;0, "F", D14=0, "-")</f>
@@ -13909,7 +13908,7 @@
       </c>
       <c r="B15" s="131">
         <f>B14*(1-B17)</f>
-        <v>46045.650000000009</v>
+        <v>46105.650000000009</v>
       </c>
       <c r="C15" s="131">
         <f>C14*0.3</f>
@@ -13917,11 +13916,11 @@
       </c>
       <c r="D15" s="131">
         <f t="shared" si="1"/>
-        <v>-260.59524999999121</v>
+        <v>-200.59524999999121</v>
       </c>
       <c r="E15" s="132">
         <f t="shared" si="2"/>
-        <v>-5.6276480330693657E-3</v>
+        <v>-4.3319264802622603E-3</v>
       </c>
       <c r="F15" s="130" t="str" cm="1">
         <f t="array" ref="F15">_xlfn.IFS(D15&gt;0, "U", D15&lt;0, "F", D15=0, "-")</f>
@@ -13937,7 +13936,7 @@
       </c>
       <c r="B16" s="146">
         <f>B14-B15</f>
-        <v>107439.84999999999</v>
+        <v>107579.84999999999</v>
       </c>
       <c r="C16" s="146">
         <f>C14-C15</f>
@@ -13945,11 +13944,11 @@
       </c>
       <c r="D16" s="146">
         <f t="shared" si="1"/>
-        <v>-608.0555833333492</v>
+        <v>-468.0555833333492</v>
       </c>
       <c r="E16" s="147">
         <f t="shared" si="2"/>
-        <v>-5.6276480330696987E-3</v>
+        <v>-4.3319264802625934E-3</v>
       </c>
       <c r="F16" s="148" t="str" cm="1">
         <f t="array" ref="F16">_xlfn.IFS(D16&lt;0, "U", D16&gt;0, "F", D16=0, "-")</f>
@@ -14101,7 +14100,7 @@
       </c>
       <c r="B22" s="152">
         <f>B16-B21</f>
-        <v>34439.849999999991</v>
+        <v>34579.849999999991</v>
       </c>
       <c r="C22" s="152">
         <f>C16-C21</f>
@@ -14109,11 +14108,11 @@
       </c>
       <c r="D22" s="152">
         <f t="shared" si="1"/>
-        <v>391.9444166666508</v>
+        <v>531.9444166666508</v>
       </c>
       <c r="E22" s="153">
         <f t="shared" si="2"/>
-        <v>1.1511557317596344E-2</v>
+        <v>1.5623410825218009E-2</v>
       </c>
       <c r="F22" s="154" t="str" cm="1">
         <f t="array" ref="F22">_xlfn.IFS(D22&lt;0, "U", D22&gt;0, "F", D22=0, "-")</f>
@@ -14129,7 +14128,7 @@
       </c>
       <c r="B23" s="162">
         <f>B22/B14</f>
-        <v>0.22438503962915057</v>
+        <v>0.22500398541176617</v>
       </c>
       <c r="C23" s="162">
         <f>C22/C14</f>
@@ -14137,11 +14136,11 @@
       </c>
       <c r="D23" s="132">
         <f t="shared" si="1"/>
-        <v>3.8020141678063168E-3</v>
+        <v>4.4209599504219099E-3</v>
       </c>
       <c r="E23" s="132">
         <f t="shared" si="2"/>
-        <v>1.7236204643827469E-2</v>
+        <v>2.0042158462445503E-2</v>
       </c>
       <c r="F23" s="130" t="str" cm="1">
         <f t="array" ref="F23">IFERROR(_xlfn.IFS(D23&lt;0, "U", D23&gt;0, "F", D23=0, "-"), "-")</f>
@@ -14178,8 +14177,8 @@
         <v>42</v>
       </c>
       <c r="C30" s="123">
-        <f>IFERROR(B30-_xlfn.XLOOKUP("Active Customers",'KPI Tracker'!$A$4:$A$16,'KPI Tracker'!$B$4:$B$16),"—")</f>
-        <v>3</v>
+        <f>IFERROR(B30-_xlfn.XLOOKUP("Active Customers",'KPI Tracker'!$A$4:$A$16,'KPI Tracker'!$C$4:$C$16),"—")</f>
+        <v>1</v>
       </c>
       <c r="D30" s="123" t="s">
         <v>678</v>
@@ -14192,9 +14191,9 @@
       <c r="B31" s="161">
         <v>54</v>
       </c>
-      <c r="C31" s="123" t="str">
-        <f>IFERROR(B31-_xlfn.XLOOKUP("Active Subscriptions",'KPI Tracker'!$A$4:$A$16,'KPI Tracker'!$B$4:$B$16),"—")</f>
-        <v>—</v>
+      <c r="C31" s="123">
+        <f>B31-'Feb 2026 A vs F'!B31</f>
+        <v>1</v>
       </c>
       <c r="D31" s="123" t="s">
         <v>679</v>
@@ -14209,11 +14208,11 @@
       </c>
       <c r="B32" s="131">
         <f>B9/B30</f>
-        <v>3654.4166666666665</v>
+        <v>3659.1785714285716</v>
       </c>
       <c r="C32" s="131">
-        <f>IFERROR(B32-_xlfn.XLOOKUP("ARPA",'KPI Tracker'!$A$4:$A$16,'KPI Tracker'!$B$4:$B$16),"—")</f>
-        <v>-57.878205128205082</v>
+        <f>B32-'Feb 2026 A vs F'!B32</f>
+        <v>-6.8092334494772331</v>
       </c>
       <c r="D32" s="123" t="s">
         <v>617</v>
@@ -14228,7 +14227,7 @@
         <v>0.7</v>
       </c>
       <c r="C33" s="162">
-        <f>IFERROR(B33-_xlfn.XLOOKUP("Gross Margin",'KPI Tracker'!$A$4:$A$16,'KPI Tracker'!$B$4:$B$16),"—")</f>
+        <f>B33-'Feb 2026 A vs F'!B33</f>
         <v>0</v>
       </c>
       <c r="D33" s="123" t="s">
@@ -14240,12 +14239,12 @@
         <v>620</v>
       </c>
       <c r="B34" s="162">
-        <f>Retention!AA6</f>
-        <v>0.99610819735501566</v>
+        <f>Retention!AB6</f>
+        <v>1</v>
       </c>
       <c r="C34" s="162">
-        <f>IFERROR(B34-_xlfn.XLOOKUP("GRR",'KPI Tracker'!$A$4:$A$16,'KPI Tracker'!$B$4:$B$16),"—")</f>
-        <v>-3.8918026449843435E-3</v>
+        <f>B34-'Feb 2026 A vs F'!B34</f>
+        <v>3.8918026449843435E-3</v>
       </c>
       <c r="D34" s="123" t="s">
         <v>621</v>
@@ -14256,12 +14255,12 @@
         <v>622</v>
       </c>
       <c r="B35" s="162">
-        <f>Retention!AA7</f>
-        <v>0.99610819735501566</v>
+        <f>Retention!AB7</f>
+        <v>1.00240271380201</v>
       </c>
       <c r="C35" s="162">
-        <f>IFERROR(B35-_xlfn.XLOOKUP("NRR",'KPI Tracker'!$A$4:$A$16,'KPI Tracker'!$B$4:$B$16),"—")</f>
-        <v>-3.8918026449843435E-3</v>
+        <f>B35-'Feb 2026 A vs F'!B35</f>
+        <v>6.2945164469943027E-3</v>
       </c>
       <c r="D35" s="123" t="s">
         <v>621</v>
@@ -14292,8 +14291,8 @@
         <v>29000</v>
       </c>
       <c r="C37" s="163">
-        <f>IFERROR(B37-_xlfn.XLOOKUP("S&amp;M (actual)",'KPI Tracker'!$A$4:$A$16,'KPI Tracker'!$B$4:$B$16),"—")</f>
-        <v>-1000</v>
+        <f>B37-'Feb 2026 A vs F'!B37</f>
+        <v>-2000</v>
       </c>
       <c r="D37" s="123" t="s">
         <v>626</v>
@@ -14308,8 +14307,8 @@
         <v>14500</v>
       </c>
       <c r="C38" s="163">
-        <f>IFERROR(IF(ISNUMBER(B38),B38-_xlfn.XLOOKUP("CAC — monthly",'KPI Tracker'!$A$4:$A$16,'KPI Tracker'!$B$4:$B$16),"—"),"—")</f>
-        <v>-15500</v>
+        <f>B38-'Feb 2026 A vs F'!B38</f>
+        <v>-1000</v>
       </c>
       <c r="D38" s="123" t="s">
         <v>662</v>
@@ -14343,7 +14342,7 @@
       <c r="D40" s="123" t="s">
         <v>663</v>
       </c>
-      <c r="K40" s="217"/>
+      <c r="K40" s="211"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="123" t="s">
@@ -14429,11 +14428,11 @@
       </c>
       <c r="B54" s="131">
         <f>B32</f>
-        <v>3654.4166666666665</v>
+        <v>3659.1785714285716</v>
       </c>
       <c r="C54" s="131">
         <f>B9/B30</f>
-        <v>3654.4166666666665</v>
+        <v>3659.1785714285716</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
@@ -14442,7 +14441,7 @@
       </c>
       <c r="B55" s="162">
         <f>B34</f>
-        <v>0.99610819735501566</v>
+        <v>1</v>
       </c>
       <c r="C55" s="162">
         <f>Retention!AA6</f>
@@ -14455,7 +14454,7 @@
       </c>
       <c r="B56" s="162">
         <f>B35</f>
-        <v>0.99610819735501566</v>
+        <v>1.00240271380201</v>
       </c>
       <c r="C56" s="162">
         <f>Retention!AA7</f>
@@ -14494,32 +14493,32 @@
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A61" s="218" t="s">
+      <c r="A61" s="212" t="s">
         <v>722</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A62" s="218" t="s">
+      <c r="A62" s="212" t="s">
         <v>719</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A63" s="218" t="s">
+      <c r="A63" s="212" t="s">
         <v>720</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A64" s="218" t="s">
+      <c r="A64" s="212" t="s">
         <v>721</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A66" s="198" t="s">
+      <c r="A66" s="193" t="s">
         <v>697</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A68" s="199" t="s">
+      <c r="A68" s="194" t="s">
         <v>698</v>
       </c>
     </row>
@@ -14535,7 +14534,7 @@
       <c r="A70" s="126" t="s">
         <v>700</v>
       </c>
-      <c r="B70" s="200">
+      <c r="B70" s="195">
         <f>'Jan 2026 A vs F '!B4+'Feb 2026 A vs F'!B4+'Mar 2026 A vs F'!B4</f>
         <v>10830</v>
       </c>
@@ -14544,16 +14543,16 @@
       <c r="A71" s="126" t="s">
         <v>701</v>
       </c>
-      <c r="B71" s="200">
+      <c r="B71" s="195">
         <f>'Jan 2026 A vs F '!B5+'Feb 2026 A vs F'!B5+'Mar 2026 A vs F'!B5</f>
-        <v>180</v>
+        <v>380</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" s="126" t="s">
         <v>702</v>
       </c>
-      <c r="B72" s="200">
+      <c r="B72" s="195">
         <f>'Jan 2026 A vs F '!B7+'Feb 2026 A vs F'!B7+'Mar 2026 A vs F'!B7</f>
         <v>594</v>
       </c>
@@ -14562,22 +14561,22 @@
       <c r="A73" s="126" t="s">
         <v>703</v>
       </c>
-      <c r="B73" s="200">
+      <c r="B73" s="195">
         <f>'Jan 2026 A vs F '!B8+'Feb 2026 A vs F'!B8+'Mar 2026 A vs F'!B8</f>
-        <v>10416</v>
+        <v>10616</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" s="127" t="s">
         <v>146</v>
       </c>
-      <c r="B74" s="201">
+      <c r="B74" s="196">
         <f>'Mar 2026 A vs F'!B9</f>
-        <v>153485.5</v>
+        <v>153685.5</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A76" s="199" t="s">
+      <c r="A76" s="194" t="s">
         <v>704</v>
       </c>
     </row>
@@ -14593,9 +14592,9 @@
       <c r="A78" s="126" t="s">
         <v>706</v>
       </c>
-      <c r="B78" s="200">
+      <c r="B78" s="195">
         <f>'Jan 2026 A vs F '!B14+'Feb 2026 A vs F'!B14+'Mar 2026 A vs F'!B14</f>
-        <v>448570.5</v>
+        <v>448770.5</v>
       </c>
       <c r="C78" s="30"/>
     </row>
@@ -14603,25 +14602,25 @@
       <c r="A79" s="126" t="s">
         <v>707</v>
       </c>
-      <c r="B79" s="200">
+      <c r="B79" s="195">
         <f>'Jan 2026 A vs F '!B15+'Feb 2026 A vs F'!B15+'Mar 2026 A vs F'!B15</f>
-        <v>134571.15000000002</v>
+        <v>134631.15000000002</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" s="127" t="s">
         <v>708</v>
       </c>
-      <c r="B80" s="201">
+      <c r="B80" s="196">
         <f>B78-B79</f>
-        <v>313999.34999999998</v>
+        <v>314139.34999999998</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" s="126" t="s">
         <v>709</v>
       </c>
-      <c r="B81" s="202">
+      <c r="B81" s="197">
         <f>B80/B78</f>
         <v>0.7</v>
       </c>
@@ -14630,7 +14629,7 @@
       <c r="A82" s="126" t="s">
         <v>710</v>
       </c>
-      <c r="B82" s="200">
+      <c r="B82" s="195">
         <f>'Jan 2026 A vs F '!B18+'Feb 2026 A vs F'!B18+'Mar 2026 A vs F'!B18</f>
         <v>90000</v>
       </c>
@@ -14639,7 +14638,7 @@
       <c r="A83" s="126" t="s">
         <v>711</v>
       </c>
-      <c r="B83" s="200">
+      <c r="B83" s="195">
         <f>'Jan 2026 A vs F '!B19+'Jan 2026 A vs F '!B20+'Feb 2026 A vs F'!B19+'Feb 2026 A vs F'!B20+'Mar 2026 A vs F'!B19+'Mar 2026 A vs F'!B20</f>
         <v>132000</v>
       </c>
@@ -14648,7 +14647,7 @@
       <c r="A84" s="127" t="s">
         <v>712</v>
       </c>
-      <c r="B84" s="201">
+      <c r="B84" s="196">
         <f>'Jan 2026 A vs F '!B21+'Feb 2026 A vs F'!B21+'Mar 2026 A vs F'!B21</f>
         <v>222000</v>
       </c>
@@ -14657,27 +14656,27 @@
       <c r="A85" s="127" t="s">
         <v>713</v>
       </c>
-      <c r="B85" s="201">
+      <c r="B85" s="196">
         <f>B80-B84</f>
-        <v>91999.349999999977</v>
+        <v>92139.349999999977</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A86" s="126" t="s">
         <v>714</v>
       </c>
-      <c r="B86" s="202">
+      <c r="B86" s="197">
         <f>B85/B78</f>
-        <v>0.2050945169154012</v>
+        <v>0.20531507752849168</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A88" s="199" t="s">
+      <c r="A88" s="194" t="s">
         <v>715</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A89" s="203" t="s">
+      <c r="A89" s="198" t="s">
         <v>4</v>
       </c>
       <c r="B89" s="125" t="s">
@@ -14689,8 +14688,8 @@
         <v>716</v>
       </c>
       <c r="B90" s="120">
-        <f>B30-'KPI Tracker'!B5</f>
-        <v>3</v>
+        <f>1+('Feb 2026 A vs F'!B30-'Jan 2026 A vs F '!B39)+'Mar 2026 A vs F'!B39</f>
+        <v>5</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.35">
@@ -14699,7 +14698,7 @@
       </c>
       <c r="B91" s="100">
         <f>B82/B90</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.35">
@@ -14708,49 +14707,49 @@
       </c>
       <c r="B92" s="100">
         <f>(B81/((B72/'Jan 2026 A vs F '!B3)*12)*'Mar 2026 A vs F'!B54)</f>
-        <v>51344.682337846047</v>
+        <v>51411.587266764865</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>631</v>
       </c>
-      <c r="B93" s="204">
+      <c r="B93" s="199">
         <f>B92/B91</f>
-        <v>1.7114894112615349</v>
+        <v>2.8561992925980482</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>718</v>
       </c>
-      <c r="B94" s="204">
+      <c r="B94" s="199">
         <f>B91/(B54*B81)</f>
-        <v>11.727492173527795</v>
+        <v>7.0273382980177059</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A96" s="216" t="s">
+      <c r="A96" s="210" t="s">
         <v>723</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A97" s="218" t="s">
+      <c r="A97" s="212" t="s">
         <v>724</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A98" s="218" t="s">
+      <c r="A98" s="212" t="s">
         <v>725</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A99" s="218" t="s">
+      <c r="A99" s="212" t="s">
         <v>726</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A100" s="218" t="s">
+      <c r="A100" s="212" t="s">
         <v>727</v>
       </c>
     </row>
@@ -15684,11 +15683,11 @@
       </c>
       <c r="D4" s="131">
         <f>'Mar 2026 A vs F'!B9</f>
-        <v>153485.5</v>
-      </c>
-      <c r="E4" s="205">
+        <v>153685.5</v>
+      </c>
+      <c r="E4" s="174">
         <f>'Mar 2026 A vs F'!B74</f>
-        <v>153485.5</v>
+        <v>153685.5</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -15707,7 +15706,7 @@
         <f>'Mar 2026 A vs F'!B30</f>
         <v>42</v>
       </c>
-      <c r="E5" s="206">
+      <c r="E5" s="200">
         <f>'Mar 2026 A vs F'!B30</f>
         <v>42</v>
       </c>
@@ -15726,11 +15725,11 @@
       </c>
       <c r="D6" s="131">
         <f>'Mar 2026 A vs F'!B32</f>
-        <v>3654.4166666666665</v>
-      </c>
-      <c r="E6" s="205">
+        <v>3659.1785714285716</v>
+      </c>
+      <c r="E6" s="174">
         <f>'Mar 2026 A vs F'!B74/'Mar 2026 A vs F'!B30</f>
-        <v>3654.4166666666665</v>
+        <v>3659.1785714285716</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -15749,7 +15748,7 @@
         <f>'Mar 2026 A vs F'!B33</f>
         <v>0.7</v>
       </c>
-      <c r="E7" s="207">
+      <c r="E7" s="201">
         <f>'Mar 2026 A vs F'!B81</f>
         <v>0.7</v>
       </c>
@@ -15768,11 +15767,11 @@
       </c>
       <c r="D8" s="162">
         <f>'Mar 2026 A vs F'!B34</f>
-        <v>0.99610819735501566</v>
-      </c>
-      <c r="E8" s="208">
+        <v>1</v>
+      </c>
+      <c r="E8" s="202">
         <f>'Mar 2026 A vs F'!B34</f>
-        <v>0.99610819735501566</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -15789,11 +15788,11 @@
       </c>
       <c r="D9" s="162">
         <f>'Mar 2026 A vs F'!B35</f>
-        <v>0.99610819735501566</v>
-      </c>
-      <c r="E9" s="207">
+        <v>1.00240271380201</v>
+      </c>
+      <c r="E9" s="201">
         <f>'Mar 2026 A vs F'!B35</f>
-        <v>0.99610819735501566</v>
+        <v>1.00240271380201</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -15808,7 +15807,7 @@
         <f>'Mar 2026 A vs F'!B36</f>
         <v>N/A — no losses</v>
       </c>
-      <c r="E10" s="209" t="s">
+      <c r="E10" s="203" t="s">
         <v>629</v>
       </c>
     </row>
@@ -15828,7 +15827,7 @@
         <f>'Mar 2026 A vs F'!B37</f>
         <v>29000</v>
       </c>
-      <c r="E11" s="210">
+      <c r="E11" s="204">
         <f>'Mar 2026 A vs F'!B82</f>
         <v>90000</v>
       </c>
@@ -15849,9 +15848,9 @@
         <f>'Mar 2026 A vs F'!B38</f>
         <v>14500</v>
       </c>
-      <c r="E12" s="211">
+      <c r="E12" s="205">
         <f>'Mar 2026 A vs F'!B91</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -15863,9 +15862,9 @@
       </c>
       <c r="C13" s="121"/>
       <c r="D13" s="121"/>
-      <c r="E13" s="212">
+      <c r="E13" s="206">
         <f>'Mar 2026 A vs F'!B91</f>
-        <v>30000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -15877,9 +15876,9 @@
       </c>
       <c r="C14" s="121"/>
       <c r="D14" s="121"/>
-      <c r="E14" s="213">
+      <c r="E14" s="207">
         <f>'Mar 2026 A vs F'!B92</f>
-        <v>51344.682337846047</v>
+        <v>51411.587266764865</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -15891,9 +15890,9 @@
       </c>
       <c r="C15" s="121"/>
       <c r="D15" s="121"/>
-      <c r="E15" s="214">
+      <c r="E15" s="208">
         <f>'Mar 2026 A vs F'!B93</f>
-        <v>1.7114894112615349</v>
+        <v>2.8561992925980482</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -15905,17 +15904,17 @@
       </c>
       <c r="C16" s="121"/>
       <c r="D16" s="121"/>
-      <c r="E16" s="215">
+      <c r="E16" s="209">
         <f>'Mar 2026 A vs F'!B94</f>
-        <v>11.727492173527795</v>
+        <v>7.0273382980177059</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="194" t="s">
+      <c r="A18" s="214" t="s">
         <v>644</v>
       </c>
-      <c r="B18" s="194"/>
-      <c r="C18" s="194"/>
+      <c r="B18" s="214"/>
+      <c r="C18" s="214"/>
       <c r="D18" s="122"/>
       <c r="E18" s="122"/>
     </row>
@@ -16300,7 +16299,7 @@
       </c>
       <c r="C18" s="184">
         <f>'Mar 2026 A vs F'!B5</f>
-        <v>180</v>
+        <v>380</v>
       </c>
       <c r="D18" s="184">
         <f>'Mar 2026 A vs F'!C5</f>
@@ -16308,7 +16307,7 @@
       </c>
       <c r="E18" s="179">
         <f>'Mar 2026 A vs F'!D5</f>
-        <v>-535.34749999999997</v>
+        <v>-335.34749999999997</v>
       </c>
       <c r="I18" t="s">
         <v>668</v>
@@ -16366,7 +16365,7 @@
       </c>
       <c r="C21" s="185">
         <f>'Mar 2026 A vs F'!B8</f>
-        <v>3180</v>
+        <v>3380</v>
       </c>
       <c r="D21" s="185">
         <f>'Mar 2026 A vs F'!C8</f>
@@ -16374,7 +16373,7 @@
       </c>
       <c r="E21" s="183">
         <f>'Mar 2026 A vs F'!D8</f>
-        <v>-581.55083333333323</v>
+        <v>-381.55083333333323</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
@@ -16387,7 +16386,7 @@
       </c>
       <c r="C22" s="181">
         <f>'Mar 2026 A vs F'!B9</f>
-        <v>153485.5</v>
+        <v>153685.5</v>
       </c>
       <c r="D22" s="181">
         <f>'Mar 2026 A vs F'!C9</f>
@@ -16395,7 +16394,7 @@
       </c>
       <c r="E22" s="180">
         <f>'Mar 2026 A vs F'!D9</f>
-        <v>-868.65083333334769</v>
+        <v>-668.65083333334769</v>
       </c>
     </row>
   </sheetData>

</xml_diff>